<commit_message>
Pruebo horario especifico con branch correcta
</commit_message>
<xml_diff>
--- a/github_actions/automatize_predict/schedules.xlsx
+++ b/github_actions/automatize_predict/schedules.xlsx
@@ -451,90 +451,90 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45462.85416666666</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="B2" t="n">
         <v>167</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45462.84375</v>
+        <v>45462.96875</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45462.86458333334</v>
+        <v>45462.98958333334</v>
       </c>
       <c r="B3" t="n">
         <v>167</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45462.85416666666</v>
+        <v>45462.97916666666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45462.89583333334</v>
+        <v>45463.02083333334</v>
       </c>
       <c r="B4" t="n">
         <v>167</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45462.88541666666</v>
+        <v>45463.01041666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45462.97916666666</v>
+        <v>45463.10416666666</v>
       </c>
       <c r="B5" t="n">
         <v>167</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45462.96875</v>
+        <v>45463.09375</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45465.85416666666</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="B6" t="n">
         <v>167</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45465.84375</v>
+        <v>45465.96875</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45465.89583333334</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="B7" t="n">
         <v>167</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45465.88541666666</v>
+        <v>45466.01041666666</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45465.9375</v>
+        <v>45466.0625</v>
       </c>
       <c r="B8" t="n">
         <v>167</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45465.92708333334</v>
+        <v>45466.05208333334</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.10416666666</v>
       </c>
       <c r="B9" t="n">
         <v>167</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45465.96875</v>
+        <v>45466.09375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>